<commit_message>
adding readme and changes to scripts
</commit_message>
<xml_diff>
--- a/Extra files/inventory_simulation_daily_detailed_1s.xlsx
+++ b/Extra files/inventory_simulation_daily_detailed_1s.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristineandersen/Desktop/Speciale/Thesis_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristineandersen/Desktop/Speciale/Thesis_project/Extra files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{081BC11C-7DBF-6E40-8256-C013682F1CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653118D2-E29E-AD4E-830B-98E2F94C7250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="880" windowWidth="28040" windowHeight="16940" xr2:uid="{12355749-DCC8-6049-92D8-2AAA63248AC6}"/>
+    <workbookView xWindow="300" yWindow="880" windowWidth="28040" windowHeight="16940" xr2:uid="{12355749-DCC8-6049-92D8-2AAA63248AC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -4244,7 +4244,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Average of ordered_today</t>
+    <t>StdDev of ordered_today</t>
   </si>
 </sst>
 </file>
@@ -22894,7 +22894,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC488C46-4FBC-4240-BDBA-C63C83945CE6}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC488C46-4FBC-4240-BDBA-C63C83945CE6}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="23">
     <pivotField numFmtId="14" showAll="0"/>
@@ -22969,7 +22969,7 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Average of ordered_today" fld="14" subtotal="average" baseField="0" baseItem="0"/>
+    <dataField name="StdDev of ordered_today" fld="14" subtotal="stdDev" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -23304,7 +23304,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -23320,7 +23320,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="5">
-        <v>98.62222222222222</v>
+        <v>38.716943936928075</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -23328,7 +23328,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="5">
-        <v>99.077777777777783</v>
+        <v>36.00100740718355</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -23336,7 +23336,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="5">
-        <v>100.2</v>
+        <v>40.608074693798017</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -23344,7 +23344,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="5">
-        <v>97.522222222222226</v>
+        <v>37.947103271417639</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -23352,7 +23352,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="5">
-        <v>94.444444444444443</v>
+        <v>39.303804061856837</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -23360,7 +23360,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="5">
-        <v>93.13333333333334</v>
+        <v>40.011571360003217</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -23368,7 +23368,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="5">
-        <v>92.077777777777783</v>
+        <v>40.791667957825929</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -23376,7 +23376,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="5">
-        <v>95.655555555555551</v>
+        <v>40.5277436146756</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -23384,7 +23384,7 @@
         <v>1404</v>
       </c>
       <c r="B12" s="5">
-        <v>96.341666666666669</v>
+        <v>39.175471839920313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>